<commit_message>
Fix: Preserve leading zeros in NISN and contact fields - Set Excel columns B & C as TEXT format in template generation - Change Siswa model cast from integer to string for NISN - Add monospace font style to all NISN/contact displays - Update import logic to handle TEXT format properly - Add logo fallback paths for PDF generation - Add check-logo.php diagnostic tool
</commit_message>
<xml_diff>
--- a/public/templates/template_import_siswa.xlsx
+++ b/public/templates/template_import_siswa.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="32">
   <si>
     <t>Nama</t>
   </si>
@@ -44,7 +44,7 @@
     <t>081234567890</t>
   </si>
   <si>
-    <t>IPA</t>
+    <t>Teknologi Komputer Jaringan</t>
   </si>
   <si>
     <t>Ani Putri</t>
@@ -56,16 +56,7 @@
     <t>081298765432</t>
   </si>
   <si>
-    <t>IPS</t>
-  </si>
-  <si>
-    <t>Ahmad Zaki</t>
-  </si>
-  <si>
-    <t>0051234569</t>
-  </si>
-  <si>
-    <t>081345678901</t>
+    <t>Akuntansi</t>
   </si>
   <si>
     <t>KETERANGAN:</t>
@@ -77,15 +68,18 @@
     <t>- NISN: Nomor Induk Siswa Nasional (wajib, harus unik, 10-20 digit)</t>
   </si>
   <si>
-    <t xml:space="preserve">  PENTING: NISN sudah otomatis diformat TEXT di template ini!</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Jangan ubah format kolom NISN agar angka 0 di depan tidak hilang</t>
+    <t xml:space="preserve">  Kolom ini sudah di-set sebagai TEXT, cukup ketik angka saja: 0051234567</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Angka 0 di depan akan tetap tersimpan</t>
   </si>
   <si>
     <t>- Kontak Ortu: Nomor HP orang tua (opsional)</t>
   </si>
   <si>
+    <t xml:space="preserve">  Kolom ini sudah TEXT, ketik langsung: 081234567890</t>
+  </si>
+  <si>
     <t>- Kelas: Angka kelas: 10, 11, atau 12 (wajib)</t>
   </si>
   <si>
@@ -101,19 +95,22 @@
     <t>CARA MENGGUNAKAN:</t>
   </si>
   <si>
-    <t>1. Hapus 3 baris contoh data (baris 2-4)</t>
+    <t>1. Hapus 2 baris contoh data (baris 2-3)</t>
   </si>
   <si>
     <t>2. Isi data siswa mulai dari baris 2</t>
   </si>
   <si>
-    <t>3. Pastikan kombinasi Kelas dan Jurusan sudah ada di database!</t>
-  </si>
-  <si>
-    <t>4. NISN harus unik dan belum terdaftar</t>
-  </si>
-  <si>
-    <t>5. Simpan file dan upload di menu Import Excel</t>
+    <t>3. Ketik NISN dan Kontak Ortu langsung (TIDAK perlu tanda petik ')</t>
+  </si>
+  <si>
+    <t>4. Pastikan kombinasi Kelas dan Jurusan sudah ada di database!</t>
+  </si>
+  <si>
+    <t>5. NISN harus unik dan belum terdaftar</t>
+  </si>
+  <si>
+    <t>6. Simpan file dan upload di menu Import Excel</t>
   </si>
 </sst>
 </file>
@@ -191,11 +188,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
     <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
+    <xf xfId="0" fontId="1" numFmtId="49" fillId="2" borderId="1" applyFont="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="0" numFmtId="49" fillId="0" borderId="0" applyFont="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="0"/>
     <xf xfId="0" fontId="2" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -496,12 +497,12 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="true" style="0"/>
-    <col min="2" max="2" width="15" customWidth="true" style="0"/>
-    <col min="3" max="3" width="15" customWidth="true" style="0"/>
+    <col min="2" max="2" width="15" customWidth="true" style="3"/>
+    <col min="3" max="3" width="15" customWidth="true" style="3"/>
     <col min="4" max="4" width="10" customWidth="true" style="0"/>
     <col min="5" max="5" width="15" customWidth="true" style="0"/>
     <col min="6" max="6" width="15" customWidth="true" style="0"/>
@@ -511,10 +512,10 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
@@ -531,10 +532,10 @@
       <c r="A2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D2">
@@ -544,17 +545,17 @@
         <v>9</v>
       </c>
       <c r="F2">
-        <v>2024</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
         <v>10</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="3" t="s">
         <v>12</v>
       </c>
       <c r="D3">
@@ -564,77 +565,62 @@
         <v>13</v>
       </c>
       <c r="F3">
-        <v>2024</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
-      <c r="A4" t="s">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B4" t="s">
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" t="s">
         <v>15</v>
-      </c>
-      <c r="C4" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4">
-        <v>11</v>
-      </c>
-      <c r="E4" t="s">
-        <v>9</v>
-      </c>
-      <c r="F4">
-        <v>2023</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
-      <c r="A6" s="2" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -642,36 +628,42 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="22" spans="1:6">
       <c r="A22" t="s">
-        <v>32</v>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
+      <c r="A23" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>
   <mergeCells>
+    <mergeCell ref="A6:F6"/>
     <mergeCell ref="A7:F7"/>
     <mergeCell ref="A8:F8"/>
     <mergeCell ref="A9:F9"/>
@@ -688,6 +680,7 @@
     <mergeCell ref="A20:F20"/>
     <mergeCell ref="A21:F21"/>
     <mergeCell ref="A22:F22"/>
+    <mergeCell ref="A23:F23"/>
   </mergeCells>
   <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>